<commit_message>
auto: actualizar indicadores adelantados 2026-09-14
</commit_message>
<xml_diff>
--- a/datos/indicadores_adelantados/cemento/consumo_cemento_depto_2000_2026.xlsx
+++ b/datos/indicadores_adelantados/cemento/consumo_cemento_depto_2000_2026.xlsx
@@ -1,25 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24332"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\3. IGAE\2026-08 Agosto\5. Cemento\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\1. Página Web\2026 - 09. Septiembre\Cemento 6-2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{342EFA19-0BBB-4E12-96A3-44759F924A96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="11565" windowHeight="11010"/>
+    <workbookView xWindow="-28920" yWindow="-75" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="C3" sheetId="2" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029" iterate="1" iterateCount="1000" calcOnSave="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="29">
   <si>
     <t>PERIODO</t>
   </si>
@@ -182,7 +183,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="0.0000000"/>
@@ -685,6 +686,23 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
@@ -720,6 +738,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -895,7 +930,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B1:Q383"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -13486,44 +13521,44 @@
         <v>27</v>
       </c>
       <c r="C370" s="19">
-        <f>SUM(C371:C376)</f>
-        <v>161985.94</v>
+        <f>SUM(C371:C377)</f>
+        <v>195167.29</v>
       </c>
       <c r="D370" s="19">
-        <f t="shared" ref="D370:K370" si="0">SUM(D371:D376)</f>
-        <v>312062.12799999991</v>
+        <f t="shared" ref="D370:K370" si="0">SUM(D371:D377)</f>
+        <v>377662.1779999999</v>
       </c>
       <c r="E370" s="19">
         <f t="shared" si="0"/>
-        <v>325965.56999999989</v>
+        <v>420016.8299999999</v>
       </c>
       <c r="F370" s="19">
         <f t="shared" si="0"/>
-        <v>70725.11</v>
+        <v>90244.760000000009</v>
       </c>
       <c r="G370" s="19">
         <f t="shared" si="0"/>
-        <v>57205.049999999996</v>
+        <v>66894.95</v>
       </c>
       <c r="H370" s="19">
         <f t="shared" si="0"/>
-        <v>66415.279999999897</v>
+        <v>79302.264999999898</v>
       </c>
       <c r="I370" s="19">
         <f t="shared" si="0"/>
-        <v>386576.25899999985</v>
+        <v>499977.98999999987</v>
       </c>
       <c r="J370" s="19">
         <f t="shared" si="0"/>
-        <v>18898.300000000003</v>
+        <v>23403.250000000004</v>
       </c>
       <c r="K370" s="19">
         <f t="shared" si="0"/>
-        <v>4964.45</v>
+        <v>6457.45</v>
       </c>
       <c r="L370" s="19">
         <f>SUM(C370:K370)</f>
-        <v>1404798.0869999996</v>
+        <v>1759126.9629999993</v>
       </c>
       <c r="M370" s="30"/>
       <c r="N370" s="31"/>
@@ -13563,6 +13598,7 @@
         <v>570</v>
       </c>
       <c r="L371" s="18">
+        <f>SUM(C371:K371)</f>
         <v>255767.82799999983</v>
       </c>
       <c r="M371" s="30"/>
@@ -13603,6 +13639,7 @@
         <v>1050</v>
       </c>
       <c r="L372" s="18">
+        <f t="shared" ref="L372:L375" si="1">SUM(C372:K372)</f>
         <v>201091.49</v>
       </c>
       <c r="M372" s="30"/>
@@ -13643,6 +13680,7 @@
         <v>990</v>
       </c>
       <c r="L373" s="18">
+        <f t="shared" si="1"/>
         <v>255710.32</v>
       </c>
       <c r="M373" s="30"/>
@@ -13683,6 +13721,7 @@
         <v>1014.7</v>
       </c>
       <c r="L374" s="18">
+        <f t="shared" si="1"/>
         <v>258374.00999999989</v>
       </c>
       <c r="M374" s="30"/>
@@ -13723,6 +13762,7 @@
         <v>479</v>
       </c>
       <c r="L375" s="18">
+        <f t="shared" si="1"/>
         <v>210703.82999999996</v>
       </c>
       <c r="M375" s="30"/>
@@ -13754,7 +13794,7 @@
         <v>15175.2299999999</v>
       </c>
       <c r="I376" s="18">
-        <v>48651.468999999997</v>
+        <v>70147.05</v>
       </c>
       <c r="J376" s="18">
         <v>3354.65</v>
@@ -13764,7 +13804,7 @@
       </c>
       <c r="L376" s="18">
         <f>SUM(C376:K376)</f>
-        <v>223150.60899999985</v>
+        <v>244646.18999999986</v>
       </c>
       <c r="M376" s="30"/>
       <c r="N376" s="31"/>
@@ -13773,17 +13813,40 @@
       <c r="Q376" s="29"/>
     </row>
     <row r="377" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B377" s="35"/>
-      <c r="C377" s="25"/>
-      <c r="D377" s="25"/>
-      <c r="E377" s="25"/>
-      <c r="F377" s="25"/>
-      <c r="G377" s="25"/>
-      <c r="H377" s="25"/>
-      <c r="I377" s="25"/>
-      <c r="J377" s="25"/>
-      <c r="K377" s="25"/>
-      <c r="L377" s="25"/>
+      <c r="B377" s="27" t="s">
+        <v>7</v>
+      </c>
+      <c r="C377" s="18">
+        <v>33181.35</v>
+      </c>
+      <c r="D377" s="18">
+        <v>65600.05</v>
+      </c>
+      <c r="E377" s="18">
+        <v>94051.260000000009</v>
+      </c>
+      <c r="F377" s="18">
+        <v>19519.650000000001</v>
+      </c>
+      <c r="G377" s="18">
+        <v>9689.9</v>
+      </c>
+      <c r="H377" s="18">
+        <v>12886.984999999999</v>
+      </c>
+      <c r="I377" s="18">
+        <v>91906.15</v>
+      </c>
+      <c r="J377" s="18">
+        <v>4504.95</v>
+      </c>
+      <c r="K377" s="18">
+        <v>1493</v>
+      </c>
+      <c r="L377" s="18">
+        <f>SUM(C377:K377)</f>
+        <v>332833.29499999998</v>
+      </c>
       <c r="M377" s="30"/>
       <c r="N377" s="31"/>
       <c r="O377" s="28"/>
@@ -13791,23 +13854,26 @@
       <c r="Q377" s="29"/>
     </row>
     <row r="378" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B378" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="C378" s="2"/>
-      <c r="D378" s="2"/>
-      <c r="E378" s="2"/>
-      <c r="F378" s="2"/>
-      <c r="G378" s="2"/>
-      <c r="H378" s="2"/>
-      <c r="I378" s="2"/>
-      <c r="J378" s="1"/>
-      <c r="K378" s="1"/>
-      <c r="L378" s="2"/>
+      <c r="B378" s="35"/>
+      <c r="C378" s="25"/>
+      <c r="D378" s="25"/>
+      <c r="E378" s="25"/>
+      <c r="F378" s="25"/>
+      <c r="G378" s="25"/>
+      <c r="H378" s="25"/>
+      <c r="I378" s="25"/>
+      <c r="J378" s="25"/>
+      <c r="K378" s="25"/>
+      <c r="L378" s="25"/>
+      <c r="M378" s="30"/>
+      <c r="N378" s="31"/>
+      <c r="O378" s="28"/>
+      <c r="P378" s="30"/>
+      <c r="Q378" s="29"/>
     </row>
     <row r="379" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B379" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C379" s="2"/>
       <c r="D379" s="2"/>
@@ -13815,25 +13881,30 @@
       <c r="F379" s="2"/>
       <c r="G379" s="2"/>
       <c r="H379" s="2"/>
-      <c r="I379" s="1"/>
+      <c r="I379" s="2"/>
       <c r="J379" s="1"/>
       <c r="K379" s="1"/>
       <c r="L379" s="2"/>
     </row>
     <row r="380" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B380" s="26" t="s">
-        <v>23</v>
-      </c>
-      <c r="F380" s="6"/>
+      <c r="B380" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C380" s="2"/>
+      <c r="D380" s="2"/>
+      <c r="E380" s="2"/>
+      <c r="F380" s="2"/>
       <c r="G380" s="2"/>
       <c r="H380" s="2"/>
-      <c r="I380" s="2"/>
-      <c r="J380" s="2"/>
-      <c r="K380" s="2"/>
+      <c r="I380" s="1"/>
+      <c r="J380" s="1"/>
+      <c r="K380" s="1"/>
       <c r="L380" s="2"/>
     </row>
     <row r="381" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B381" s="26"/>
+      <c r="B381" s="26" t="s">
+        <v>23</v>
+      </c>
       <c r="F381" s="6"/>
       <c r="G381" s="2"/>
       <c r="H381" s="2"/>

</xml_diff>

<commit_message>
auto: actualizar datos del INE 2026-10-12
</commit_message>
<xml_diff>
--- a/datos/indicadores_adelantados/cemento/consumo_cemento_depto_2000_2026.xlsx
+++ b/datos/indicadores_adelantados/cemento/consumo_cemento_depto_2000_2026.xlsx
@@ -5,22 +5,33 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\1. Página Web\2026 - 09. Septiembre\Cemento 6-2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\1. Página Web\2026 - 10 Octubre\Cemento 8-2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{342EFA19-0BBB-4E12-96A3-44759F924A96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC4293D4-243B-4609-9E42-EBFF8A629FB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-75" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="C3" sheetId="2" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" iterate="1" iterateCount="1000" calcOnSave="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="29">
   <si>
     <t>PERIODO</t>
   </si>
@@ -931,7 +942,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:Q383"/>
+  <dimension ref="B1:Q384"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
@@ -13521,44 +13532,44 @@
         <v>27</v>
       </c>
       <c r="C370" s="19">
-        <f>SUM(C371:C377)</f>
-        <v>195167.29</v>
+        <f>SUM(C371:C378)</f>
+        <v>235509.09000000003</v>
       </c>
       <c r="D370" s="19">
-        <f t="shared" ref="D370:K370" si="0">SUM(D371:D377)</f>
-        <v>377662.1779999999</v>
+        <f t="shared" ref="D370:L370" si="0">SUM(D371:D378)</f>
+        <v>436912.2379999999</v>
       </c>
       <c r="E370" s="19">
         <f t="shared" si="0"/>
-        <v>420016.8299999999</v>
+        <v>497611.28999999992</v>
       </c>
       <c r="F370" s="19">
         <f t="shared" si="0"/>
-        <v>90244.760000000009</v>
+        <v>107994.07</v>
       </c>
       <c r="G370" s="19">
         <f t="shared" si="0"/>
-        <v>66894.95</v>
+        <v>77909.899999999994</v>
       </c>
       <c r="H370" s="19">
         <f t="shared" si="0"/>
-        <v>79302.264999999898</v>
+        <v>96556.114999999903</v>
       </c>
       <c r="I370" s="19">
         <f t="shared" si="0"/>
-        <v>499977.98999999987</v>
+        <v>574606.45999999973</v>
       </c>
       <c r="J370" s="19">
         <f t="shared" si="0"/>
-        <v>23403.250000000004</v>
+        <v>27588.800000000003</v>
       </c>
       <c r="K370" s="19">
         <f t="shared" si="0"/>
-        <v>6457.45</v>
+        <v>7342.2</v>
       </c>
       <c r="L370" s="19">
-        <f>SUM(C370:K370)</f>
-        <v>1759126.9629999993</v>
+        <f t="shared" si="0"/>
+        <v>2062030.1629999995</v>
       </c>
       <c r="M370" s="30"/>
       <c r="N370" s="31"/>
@@ -13854,17 +13865,39 @@
       <c r="Q377" s="29"/>
     </row>
     <row r="378" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B378" s="35"/>
-      <c r="C378" s="25"/>
-      <c r="D378" s="25"/>
-      <c r="E378" s="25"/>
-      <c r="F378" s="25"/>
-      <c r="G378" s="25"/>
-      <c r="H378" s="25"/>
-      <c r="I378" s="25"/>
-      <c r="J378" s="25"/>
-      <c r="K378" s="25"/>
-      <c r="L378" s="25"/>
+      <c r="B378" s="27" t="s">
+        <v>8</v>
+      </c>
+      <c r="C378" s="18">
+        <v>40341.800000000003</v>
+      </c>
+      <c r="D378" s="18">
+        <v>59250.060000000005</v>
+      </c>
+      <c r="E378" s="18">
+        <v>77594.460000000006</v>
+      </c>
+      <c r="F378" s="18">
+        <v>17749.310000000001</v>
+      </c>
+      <c r="G378" s="18">
+        <v>11014.95</v>
+      </c>
+      <c r="H378" s="18">
+        <v>17253.849999999999</v>
+      </c>
+      <c r="I378" s="18">
+        <v>74628.469999999899</v>
+      </c>
+      <c r="J378" s="18">
+        <v>4185.5499999999993</v>
+      </c>
+      <c r="K378" s="18">
+        <v>884.75</v>
+      </c>
+      <c r="L378" s="18">
+        <v>302903.1999999999</v>
+      </c>
       <c r="M378" s="30"/>
       <c r="N378" s="31"/>
       <c r="O378" s="28"/>
@@ -13872,23 +13905,26 @@
       <c r="Q378" s="29"/>
     </row>
     <row r="379" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B379" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="C379" s="2"/>
-      <c r="D379" s="2"/>
-      <c r="E379" s="2"/>
-      <c r="F379" s="2"/>
-      <c r="G379" s="2"/>
-      <c r="H379" s="2"/>
-      <c r="I379" s="2"/>
-      <c r="J379" s="1"/>
-      <c r="K379" s="1"/>
-      <c r="L379" s="2"/>
+      <c r="B379" s="35"/>
+      <c r="C379" s="25"/>
+      <c r="D379" s="25"/>
+      <c r="E379" s="25"/>
+      <c r="F379" s="25"/>
+      <c r="G379" s="25"/>
+      <c r="H379" s="25"/>
+      <c r="I379" s="25"/>
+      <c r="J379" s="25"/>
+      <c r="K379" s="25"/>
+      <c r="L379" s="25"/>
+      <c r="M379" s="30"/>
+      <c r="N379" s="31"/>
+      <c r="O379" s="28"/>
+      <c r="P379" s="30"/>
+      <c r="Q379" s="29"/>
     </row>
     <row r="380" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B380" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C380" s="2"/>
       <c r="D380" s="2"/>
@@ -13896,33 +13932,37 @@
       <c r="F380" s="2"/>
       <c r="G380" s="2"/>
       <c r="H380" s="2"/>
-      <c r="I380" s="1"/>
+      <c r="I380" s="2"/>
       <c r="J380" s="1"/>
       <c r="K380" s="1"/>
       <c r="L380" s="2"/>
     </row>
     <row r="381" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B381" s="26" t="s">
-        <v>23</v>
-      </c>
-      <c r="F381" s="6"/>
+      <c r="B381" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C381" s="2"/>
+      <c r="D381" s="2"/>
+      <c r="E381" s="2"/>
+      <c r="F381" s="2"/>
       <c r="G381" s="2"/>
       <c r="H381" s="2"/>
-      <c r="I381" s="2"/>
-      <c r="J381" s="2"/>
-      <c r="K381" s="2"/>
+      <c r="I381" s="1"/>
+      <c r="J381" s="1"/>
+      <c r="K381" s="1"/>
       <c r="L381" s="2"/>
     </row>
     <row r="382" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="C382" s="36"/>
-      <c r="D382" s="36"/>
-      <c r="E382" s="36"/>
-      <c r="F382" s="36"/>
-      <c r="G382" s="36"/>
-      <c r="H382" s="36"/>
-      <c r="I382" s="36"/>
-      <c r="J382" s="36"/>
-      <c r="K382" s="36"/>
+      <c r="B382" s="26" t="s">
+        <v>23</v>
+      </c>
+      <c r="F382" s="6"/>
+      <c r="G382" s="2"/>
+      <c r="H382" s="2"/>
+      <c r="I382" s="2"/>
+      <c r="J382" s="2"/>
+      <c r="K382" s="2"/>
+      <c r="L382" s="2"/>
     </row>
     <row r="383" spans="2:17" x14ac:dyDescent="0.25">
       <c r="C383" s="36"/>
@@ -13935,6 +13975,17 @@
       <c r="J383" s="36"/>
       <c r="K383" s="36"/>
     </row>
+    <row r="384" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="C384" s="36"/>
+      <c r="D384" s="36"/>
+      <c r="E384" s="36"/>
+      <c r="F384" s="36"/>
+      <c r="G384" s="36"/>
+      <c r="H384" s="36"/>
+      <c r="I384" s="36"/>
+      <c r="J384" s="36"/>
+      <c r="K384" s="36"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>

</xml_diff>